<commit_message>
Updated the rubric spreadsheet for the new lab 1
</commit_message>
<xml_diff>
--- a/Labs/Lab01-Review/CS233JS_Lab01_Rubric.xlsx
+++ b/Labs/Lab01-Review/CS233JS_Lab01_Rubric.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\birdb\Repos\CS233JS_Repos\CS233JS-CourseMaterials\Labs\Lab01\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Repos\CS233JS-Repos\CS233JS-CourseMaterials\Labs\Lab01-Review\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{10444EA5-CBEA-4AFD-B371-B3898A2EFE24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A5FC8B9-32BE-4F8C-8C90-E5A893173485}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="11280" xr2:uid="{5D75B731-65CD-014E-8BBA-DE69945DF98D}"/>
+    <workbookView xWindow="32760" yWindow="4572" windowWidth="18096" windowHeight="12336" activeTab="1" xr2:uid="{5D75B731-65CD-014E-8BBA-DE69945DF98D}"/>
   </bookViews>
   <sheets>
     <sheet name="Rubric" sheetId="1" r:id="rId1"/>
@@ -37,10 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="31">
-  <si>
-    <t>Possible</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="32">
   <si>
     <t>Comments</t>
   </si>
@@ -60,9 +57,6 @@
     <t>Total:</t>
   </si>
   <si>
-    <t>Web app functionality</t>
-  </si>
-  <si>
     <t>Style and best practices</t>
   </si>
   <si>
@@ -84,9 +78,6 @@
     <t>Sub-total</t>
   </si>
   <si>
-    <t>Excellent work, everything looks great!</t>
-  </si>
-  <si>
     <t>Things to look for:</t>
   </si>
   <si>
@@ -108,18 +99,6 @@
     <t>Wrong indentation</t>
   </si>
   <si>
-    <t>Paft 1: Exercises</t>
-  </si>
-  <si>
-    <t>JavaScript Quiz (based on % right)</t>
-  </si>
-  <si>
-    <t>Bootstrap tutorials (based on % completed</t>
-  </si>
-  <si>
-    <t>Part 2: Web App</t>
-  </si>
-  <si>
     <t>Completed code review form</t>
   </si>
   <si>
@@ -129,7 +108,31 @@
     <t>Lab 1: JavaScript Review &amp; Bootstrap Intro</t>
   </si>
   <si>
-    <t>Bootstrap tutorials (based on % completed)</t>
+    <t>Exercises</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paft 1: </t>
+  </si>
+  <si>
+    <t>Lab 1: JavaScript Review</t>
+  </si>
+  <si>
+    <t>Part 2: Domino Web App</t>
+  </si>
+  <si>
+    <t>No console error messages</t>
+  </si>
+  <si>
+    <t>Game works correctly</t>
+  </si>
+  <si>
+    <t>All correct</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Very good work, the game works perfectly!</t>
   </si>
 </sst>
 </file>
@@ -217,21 +220,12 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -253,7 +247,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -266,14 +260,15 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -286,10 +281,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -328,9 +319,9 @@
         </xdr:from>
         <xdr:to>
           <xdr:col>4</xdr:col>
-          <xdr:colOff>1400175</xdr:colOff>
+          <xdr:colOff>1402080</xdr:colOff>
           <xdr:row>25</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>30480</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -362,7 +353,7 @@
             </a:ln>
           </xdr:spPr>
           <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="27432" rIns="27432" bIns="27432" anchor="ctr" upright="1"/>
+            <a:bodyPr vertOverflow="clip" wrap="square" lIns="36576" tIns="32004" rIns="36576" bIns="32004" anchor="ctr" upright="1"/>
             <a:lstStyle/>
             <a:p>
               <a:pPr algn="ctr" rtl="0">
@@ -374,7 +365,6 @@
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
                   <a:latin typeface="Calibri"/>
-                  <a:ea typeface="Calibri"/>
                   <a:cs typeface="Calibri"/>
                 </a:rPr>
                 <a:t>Reset</a:t>
@@ -392,15 +382,15 @@
       <xdr:twoCellAnchor>
         <xdr:from>
           <xdr:col>4</xdr:col>
-          <xdr:colOff>180975</xdr:colOff>
+          <xdr:colOff>182880</xdr:colOff>
           <xdr:row>25</xdr:row>
           <xdr:rowOff>190500</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>4</xdr:col>
-          <xdr:colOff>1400175</xdr:colOff>
+          <xdr:colOff>1402080</xdr:colOff>
           <xdr:row>27</xdr:row>
-          <xdr:rowOff>47625</xdr:rowOff>
+          <xdr:rowOff>45720</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -432,7 +422,7 @@
             </a:ln>
           </xdr:spPr>
           <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="27432" rIns="27432" bIns="27432" anchor="ctr" upright="1"/>
+            <a:bodyPr vertOverflow="clip" wrap="square" lIns="36576" tIns="32004" rIns="36576" bIns="32004" anchor="ctr" upright="1"/>
             <a:lstStyle/>
             <a:p>
               <a:pPr algn="ctr" rtl="0">
@@ -444,7 +434,6 @@
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
                   <a:latin typeface="Calibri"/>
-                  <a:ea typeface="Calibri"/>
                   <a:cs typeface="Calibri"/>
                 </a:rPr>
                 <a:t>Add Comment</a:t>
@@ -759,74 +748,74 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7896AEF-34AA-E746-914C-B3A1A695E7D1}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:B17"/>
-  <sheetFormatPr defaultColWidth="11.125" defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr defaultColWidth="11.09765625" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="37.625" customWidth="1"/>
-    <col min="2" max="2" width="8.125" customWidth="1"/>
+    <col min="1" max="1" width="37.59765625" customWidth="1"/>
+    <col min="2" max="2" width="8.09765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.5">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.5">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="7"/>
       <c r="B3" s="7"/>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>23</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.5">
-      <c r="A5" t="s">
-        <v>24</v>
       </c>
       <c r="B5">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.5">
-      <c r="A6" t="s">
-        <v>30</v>
-      </c>
-      <c r="B6">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.5">
-      <c r="A7" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="17">
-        <f>SUM(B5:B6)</f>
-        <v>25</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.5">
-      <c r="A9" s="6" t="s">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="11">
+        <f>SUM(B5:B5)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B9" s="6"/>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.5">
+      <c r="B8" s="6"/>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="B10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>27</v>
       </c>
@@ -834,47 +823,47 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.5">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="B12">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="B13">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>8</v>
-      </c>
-      <c r="B14" s="16">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.5">
-      <c r="A15" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="B15" s="18">
-        <f>SUM(B10:B14)</f>
-        <v>25</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="16.149999999999999" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
-    <row r="17" spans="1:2" ht="16.149999999999999" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+        <v>6</v>
+      </c>
+      <c r="B14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15" s="11">
+        <f>SUM(B9:B14)</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="17" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B17" s="9">
-        <f>B7+B15</f>
-        <v>50</v>
+        <v>5</v>
+      </c>
+      <c r="B17" s="8">
+        <f>B6+B15</f>
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -885,78 +874,78 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96879333-0874-3847-ABBB-D0DF183A7724}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:E39"/>
-  <sheetFormatPr defaultColWidth="11.125" defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
+  <dimension ref="A1:F39"/>
+  <sheetFormatPr defaultColWidth="11.09765625" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="38" customWidth="1"/>
-    <col min="2" max="2" width="8" customWidth="1"/>
-    <col min="3" max="3" width="5.625" customWidth="1"/>
+    <col min="1" max="1" width="29.69921875" customWidth="1"/>
+    <col min="2" max="2" width="6.5" customWidth="1"/>
+    <col min="3" max="3" width="5.59765625" customWidth="1"/>
     <col min="4" max="4" width="1" customWidth="1"/>
-    <col min="5" max="5" width="24.125" style="4" customWidth="1"/>
-    <col min="6" max="6" width="11.125" customWidth="1"/>
+    <col min="5" max="5" width="24.09765625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="11.09765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="20.45" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:6" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.5">
-      <c r="A2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.5">
-      <c r="A3" s="15"/>
-      <c r="B3" s="15"/>
-      <c r="C3" s="15"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.5">
-      <c r="A4" s="14" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="14"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="14"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.5">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+    </row>
+    <row r="3" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="16"/>
+      <c r="B3" s="16"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="15"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>4</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>5</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="5" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="7"/>
       <c r="B6" s="7"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
-      <c r="E6" s="11"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.5">
+      <c r="E6" s="10"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" s="9"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>23</v>
-      </c>
-      <c r="E7" s="10"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.5">
-      <c r="A8" t="s">
-        <v>24</v>
       </c>
       <c r="B8">
         <v>10</v>
@@ -964,60 +953,78 @@
       <c r="C8">
         <v>10</v>
       </c>
-      <c r="E8" s="10"/>
-    </row>
-    <row r="9" spans="1:5" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A9" t="s">
-        <v>25</v>
-      </c>
-      <c r="B9">
-        <v>15</v>
-      </c>
-      <c r="C9">
-        <v>15</v>
-      </c>
-      <c r="E9" s="10"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.5">
-      <c r="A10" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" s="6">
-        <f>SUM(B8:B9)</f>
-        <v>25</v>
-      </c>
-      <c r="C10" s="6">
-        <f>SUM(C8:C9)</f>
-        <v>25</v>
-      </c>
-      <c r="E10" s="10"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.5">
+      <c r="E8" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="11">
+        <f>SUM(B8:B8)</f>
+        <v>10</v>
+      </c>
+      <c r="C9" s="11">
+        <f>SUM(C8:C8)</f>
+        <v>10</v>
+      </c>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
       <c r="D11" s="2"/>
-      <c r="E11" s="10"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.5">
-      <c r="A12" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12">
+        <v>1</v>
+      </c>
       <c r="D12" s="2"/>
-      <c r="E12" s="10"/>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.5">
+      <c r="E12" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="B13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C13">
-        <v>2</v>
-      </c>
-      <c r="E13" s="10"/>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.5">
+        <v>1</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>27</v>
       </c>
@@ -1027,159 +1034,179 @@
       <c r="C14">
         <v>2</v>
       </c>
-      <c r="E14" s="10"/>
-    </row>
-    <row r="15" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.5">
+      <c r="E14" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="F14" s="9" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="B15">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C15">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D15"/>
-      <c r="E15" s="10"/>
-    </row>
-    <row r="16" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.5">
+      <c r="E15" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="B16">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C16">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D16"/>
-      <c r="E16" s="10"/>
-    </row>
-    <row r="17" spans="1:5" s="3" customFormat="1" ht="17.45" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="E16" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" s="3" customFormat="1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>8</v>
-      </c>
-      <c r="B17" s="8">
-        <v>3</v>
-      </c>
-      <c r="C17" s="8">
-        <v>3</v>
+        <v>6</v>
+      </c>
+      <c r="B17">
+        <v>2</v>
+      </c>
+      <c r="C17">
+        <v>2</v>
       </c>
       <c r="D17" s="4"/>
-      <c r="E17" s="10"/>
-    </row>
-    <row r="18" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A18" t="s">
-        <v>14</v>
-      </c>
-      <c r="B18" s="6">
-        <f>SUM(B13:B17)</f>
-        <v>25</v>
-      </c>
-      <c r="C18" s="6">
-        <f>SUM(C13:C17)</f>
-        <v>25</v>
-      </c>
-      <c r="E18" s="10"/>
-    </row>
-    <row r="19" spans="1:5" ht="16.149999999999999" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="E17" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B18" s="11">
+        <f>SUM(B12:B17)</f>
+        <v>30</v>
+      </c>
+      <c r="C18" s="11">
+        <f>SUM(C12:C17)</f>
+        <v>30</v>
+      </c>
+      <c r="E18" s="9"/>
+    </row>
+    <row r="19" spans="1:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D19" s="2"/>
-      <c r="E19" s="10"/>
-    </row>
-    <row r="20" spans="1:5" ht="16.149999999999999" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="E19" s="9"/>
+    </row>
+    <row r="20" spans="1:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B20" s="9">
-        <f>B10+B18</f>
-        <v>50</v>
-      </c>
-      <c r="C20" s="9">
-        <f>C10+C18</f>
-        <v>50</v>
-      </c>
-      <c r="E20" s="10"/>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.5">
+        <v>5</v>
+      </c>
+      <c r="B20" s="8">
+        <f>B9+B18</f>
+        <v>40</v>
+      </c>
+      <c r="C20" s="8">
+        <f>C9+C18</f>
+        <v>40</v>
+      </c>
+      <c r="E20" s="9"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
       <c r="D24" s="3"/>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.5">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.5">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.5">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.5">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.5">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.5">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D30" s="3"/>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.5">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D31" s="1"/>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.5">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.5">
-      <c r="A34" t="s">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.5">
-      <c r="A35" t="s">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.5">
-      <c r="A36" t="s">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.5">
-      <c r="A37" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.5">
-      <c r="A38" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.5">
-      <c r="A39" t="s">
-        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -1208,9 +1235,9 @@
                   </from>
                   <to>
                     <xdr:col>4</xdr:col>
-                    <xdr:colOff>1400175</xdr:colOff>
+                    <xdr:colOff>1402080</xdr:colOff>
                     <xdr:row>25</xdr:row>
-                    <xdr:rowOff>28575</xdr:rowOff>
+                    <xdr:rowOff>30480</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -1224,15 +1251,15 @@
                 <anchor moveWithCells="1" sizeWithCells="1">
                   <from>
                     <xdr:col>4</xdr:col>
-                    <xdr:colOff>180975</xdr:colOff>
+                    <xdr:colOff>182880</xdr:colOff>
                     <xdr:row>25</xdr:row>
                     <xdr:rowOff>190500</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>4</xdr:col>
-                    <xdr:colOff>1400175</xdr:colOff>
+                    <xdr:colOff>1402080</xdr:colOff>
                     <xdr:row>27</xdr:row>
-                    <xdr:rowOff>47625</xdr:rowOff>
+                    <xdr:rowOff>45720</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>

</xml_diff>

<commit_message>
renamed old w2 notes on classes to save for archive
</commit_message>
<xml_diff>
--- a/Labs/Lab01-Review/CS233JS_Lab01_Rubric.xlsx
+++ b/Labs/Lab01-Review/CS233JS_Lab01_Rubric.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Repos\CS233JS-Repos\CS233JS-CourseMaterials\Labs\Lab01-Review\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A5FC8B9-32BE-4F8C-8C90-E5A893173485}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CF660A2-6807-4930-A9E7-0298BBDAEF96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32760" yWindow="4572" windowWidth="18096" windowHeight="12336" activeTab="1" xr2:uid="{5D75B731-65CD-014E-8BBA-DE69945DF98D}"/>
+    <workbookView xWindow="-20064" yWindow="4500" windowWidth="18096" windowHeight="12336" activeTab="1" xr2:uid="{5D75B731-65CD-014E-8BBA-DE69945DF98D}"/>
   </bookViews>
   <sheets>
     <sheet name="Rubric" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="32">
   <si>
     <t>Comments</t>
   </si>
@@ -105,9 +105,6 @@
     <t>Running correctly on citstudent</t>
   </si>
   <si>
-    <t>Lab 1: JavaScript Review &amp; Bootstrap Intro</t>
-  </si>
-  <si>
     <t>Exercises</t>
   </si>
   <si>
@@ -133,6 +130,9 @@
   </si>
   <si>
     <t>Very good work, the game works perfectly!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Part 1: </t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -773,12 +773,12 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B5">
         <v>10</v>
@@ -795,7 +795,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B8" s="6"/>
     </row>
@@ -817,7 +817,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B11">
         <v>2</v>
@@ -825,7 +825,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B12">
         <v>20</v>
@@ -887,12 +887,12 @@
   <sheetData>
     <row r="1" spans="1:6" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B2" s="14"/>
       <c r="C2" s="14"/>
@@ -939,13 +939,13 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="E7" s="9"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B8">
         <v>10</v>
@@ -954,10 +954,10 @@
         <v>10</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
@@ -981,7 +981,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>
@@ -1000,11 +1000,11 @@
         <v>1</v>
       </c>
       <c r="D12" s="2"/>
-      <c r="E12" s="9" t="s">
-        <v>30</v>
+      <c r="E12">
+        <v>1</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
@@ -1017,16 +1017,16 @@
       <c r="C13">
         <v>1</v>
       </c>
-      <c r="E13" s="9" t="s">
-        <v>30</v>
+      <c r="E13">
+        <v>1</v>
       </c>
       <c r="F13" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B14">
         <v>2</v>
@@ -1034,16 +1034,16 @@
       <c r="C14">
         <v>2</v>
       </c>
-      <c r="E14" s="9" t="s">
-        <v>30</v>
+      <c r="E14">
+        <v>2</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B15">
         <v>20</v>
@@ -1052,11 +1052,11 @@
         <v>20</v>
       </c>
       <c r="D15"/>
-      <c r="E15" s="9" t="s">
-        <v>30</v>
+      <c r="E15">
+        <v>20</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="16" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
@@ -1070,11 +1070,11 @@
         <v>4</v>
       </c>
       <c r="D16"/>
-      <c r="E16" s="9" t="s">
-        <v>30</v>
+      <c r="E16">
+        <v>4</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="17" spans="1:6" s="3" customFormat="1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
@@ -1088,11 +1088,11 @@
         <v>2</v>
       </c>
       <c r="D17" s="4"/>
-      <c r="E17" s="9" t="s">
-        <v>30</v>
+      <c r="E17">
+        <v>2</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>